<commit_message>
Add college team ranking
Roll up per-athlete totals into a college team standing. Each college's
score is the sum of every member athlete's total score, grouped
case/whitespace-insensitively and sorted highest first.

- models.py: add CollegeRanking and COLLEGE_COLUMNS (COLLEGE, ATHLETES, SCORE)
- scorer.py: add rank_colleges()
- writer.py: add a 'College Ranking' sheet
- main.py: compute rankings; add --no-colleges; log college count
- tests: add college-ranking coverage (24 tests pass)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0119jtmkdE2GaNSVKUhWNHvR
</commit_message>
<xml_diff>
--- a/examples/example_output.xlsx
+++ b/examples/example_output.xlsx
@@ -8,8 +8,9 @@
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Details" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Rejected" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="College Ranking" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Details" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Rejected" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -32,7 +33,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -43,6 +44,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F4E78"/>
         <bgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="006A1B9A"/>
+        <bgColor rgb="006A1B9A"/>
       </patternFill>
     </fill>
     <fill>
@@ -70,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -79,6 +86,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1060,6 +1070,112 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:D5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>RANK</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>COLLEGE</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>ATHLETES</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>SCORE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Fergusson College</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D2" t="n">
+        <v>9810</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>St. Xavier's</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>6</v>
+      </c>
+      <c r="D3" t="n">
+        <v>6140</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Christ University</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>4</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3813</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Loyola College</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" t="n">
+        <v>3805</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1075,47 +1191,47 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>RANK</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>NAME</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>COLLEGE</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>GENDER</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>EVENT NAME</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>PERFORMANCE TYPE</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>RESULT</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>SCORE</t>
         </is>
@@ -2158,7 +2274,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2179,47 +2295,47 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>ROW</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>NAME</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="D1" s="3" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>COLLEGE</t>
         </is>
       </c>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>GENDER</t>
         </is>
       </c>
-      <c r="F1" s="3" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>EVENT NAME</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>PERFORMANCE TYPE</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>RESULT</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>REASON</t>
         </is>

</xml_diff>